<commit_message>
Backup DB, mover arquivos ao final do processo, dedup homologação, script Telegram e verificar importações
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/data/homologacao_reabertura.xlsx
+++ b/data/homologacao_reabertura.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S62"/>
+  <dimension ref="A1:S79"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -589,27 +589,27 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>43520491826</t>
+          <t>99127563049</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>CONTROLE A PLUS - SP 24,99</t>
+          <t>TIM CONTROLE A PLUS - 31,99</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>24,99</t>
+          <t>31,99</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>11982258153</t>
+          <t>51989342461</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>11970336746</t>
+          <t>51981887224</t>
         </is>
       </c>
       <c r="F3" t="inlineStr"/>
@@ -617,12 +617,12 @@
       <c r="H3" t="inlineStr"/>
       <c r="I3" t="inlineStr">
         <is>
-          <t>1-1702518761078</t>
+          <t>1-1701716977094</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>1-1702518761078</t>
+          <t>1-1701716977094</t>
         </is>
       </c>
       <c r="K3" t="inlineStr"/>
@@ -630,12 +630,12 @@
       <c r="M3" t="inlineStr"/>
       <c r="N3" t="inlineStr">
         <is>
-          <t>250020984</t>
+          <t>250020101</t>
         </is>
       </c>
       <c r="O3" t="inlineStr">
         <is>
-          <t>250020984</t>
+          <t>250020101</t>
         </is>
       </c>
       <c r="P3" t="inlineStr"/>
@@ -650,7 +650,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>66025745072</t>
+          <t>31280601850</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -665,12 +665,12 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>51989295977</t>
+          <t>11972120276</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>51981879539</t>
+          <t>11985584636</t>
         </is>
       </c>
       <c r="F4" t="inlineStr"/>
@@ -678,12 +678,12 @@
       <c r="H4" t="inlineStr"/>
       <c r="I4" t="inlineStr">
         <is>
-          <t>1-1702407736413</t>
+          <t>1-1701262473921</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>1-1702407736413</t>
+          <t>1-1701262473921</t>
         </is>
       </c>
       <c r="K4" t="inlineStr"/>
@@ -691,12 +691,12 @@
       <c r="M4" t="inlineStr"/>
       <c r="N4" t="inlineStr">
         <is>
-          <t>250020789</t>
+          <t>250019433</t>
         </is>
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>250020789</t>
+          <t>250019433</t>
         </is>
       </c>
       <c r="P4" t="inlineStr"/>
@@ -711,7 +711,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>92079067087</t>
+          <t>28684516672</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
@@ -726,12 +726,12 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>51991652859</t>
+          <t>35998413419</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>51981887584</t>
+          <t>35991287693</t>
         </is>
       </c>
       <c r="F5" t="inlineStr"/>
@@ -739,12 +739,12 @@
       <c r="H5" t="inlineStr"/>
       <c r="I5" t="inlineStr">
         <is>
-          <t>1-1702291271693</t>
+          <t>1-1701298703548</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>1-1702291271693</t>
+          <t>1-1701298703548</t>
         </is>
       </c>
       <c r="K5" t="inlineStr"/>
@@ -752,12 +752,12 @@
       <c r="M5" t="inlineStr"/>
       <c r="N5" t="inlineStr">
         <is>
-          <t>250020700</t>
+          <t>250019293</t>
         </is>
       </c>
       <c r="O5" t="inlineStr">
         <is>
-          <t>250020700</t>
+          <t>250019293</t>
         </is>
       </c>
       <c r="P5" t="inlineStr"/>
@@ -772,7 +772,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>94162115249</t>
+          <t>17979850785</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -787,12 +787,12 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>95991241131</t>
+          <t>21995145778</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>95981277863</t>
+          <t>21982768898</t>
         </is>
       </c>
       <c r="F6" t="inlineStr"/>
@@ -800,12 +800,12 @@
       <c r="H6" t="inlineStr"/>
       <c r="I6" t="inlineStr">
         <is>
-          <t>1-1702074046684</t>
+          <t>1-1702205491001</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>1-1702074046684</t>
+          <t>1-1702205491001</t>
         </is>
       </c>
       <c r="K6" t="inlineStr"/>
@@ -813,12 +813,12 @@
       <c r="M6" t="inlineStr"/>
       <c r="N6" t="inlineStr">
         <is>
-          <t>250020429</t>
+          <t>250019221</t>
         </is>
       </c>
       <c r="O6" t="inlineStr">
         <is>
-          <t>250020429</t>
+          <t>250019221</t>
         </is>
       </c>
       <c r="P6" t="inlineStr"/>
@@ -833,7 +833,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>40163700869</t>
+          <t>36424552634</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
@@ -848,12 +848,12 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>11963206886</t>
+          <t>37999748968</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>11987378317</t>
+          <t>37991247780</t>
         </is>
       </c>
       <c r="F7" t="inlineStr"/>
@@ -861,12 +861,12 @@
       <c r="H7" t="inlineStr"/>
       <c r="I7" t="inlineStr">
         <is>
-          <t>1-1701734017039</t>
+          <t>1-1700335571847</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>1-1701734017039</t>
+          <t>1-1700335571847</t>
         </is>
       </c>
       <c r="K7" t="inlineStr"/>
@@ -874,12 +874,12 @@
       <c r="M7" t="inlineStr"/>
       <c r="N7" t="inlineStr">
         <is>
-          <t>250020156</t>
+          <t>250018415</t>
         </is>
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>250020156</t>
+          <t>250018415</t>
         </is>
       </c>
       <c r="P7" t="inlineStr"/>
@@ -894,27 +894,27 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>99127563049</t>
+          <t>50849964849</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>TIM CONTROLE A PLUS - 31,99</t>
+          <t>CONTROLE A PLUS - SP 24,99</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>31,99</t>
+          <t>24,99</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>51989342461</t>
+          <t>11942301412</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>51981887224</t>
+          <t>11983958201</t>
         </is>
       </c>
       <c r="F8" t="inlineStr"/>
@@ -922,12 +922,12 @@
       <c r="H8" t="inlineStr"/>
       <c r="I8" t="inlineStr">
         <is>
-          <t>1-1701716977094</t>
+          <t>1-1700290243600</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>1-1701716977094</t>
+          <t>1-1700290243600</t>
         </is>
       </c>
       <c r="K8" t="inlineStr"/>
@@ -935,12 +935,12 @@
       <c r="M8" t="inlineStr"/>
       <c r="N8" t="inlineStr">
         <is>
-          <t>250020101</t>
+          <t>250018145</t>
         </is>
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>250020101</t>
+          <t>250018145</t>
         </is>
       </c>
       <c r="P8" t="inlineStr"/>
@@ -955,27 +955,27 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>82833184115</t>
+          <t>35226886861</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>TIM CONTROLE A PLUS - 29,99</t>
+          <t>CONTROLE A PLUS - SP 24,99</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>29,99</t>
+          <t>24,99</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>62985830574</t>
+          <t>11995746759</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>62981531805</t>
+          <t>11983955305</t>
         </is>
       </c>
       <c r="F9" t="inlineStr"/>
@@ -983,12 +983,12 @@
       <c r="H9" t="inlineStr"/>
       <c r="I9" t="inlineStr">
         <is>
-          <t>1-1701640753773</t>
+          <t>1-1700170122242</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>1-1701640753773</t>
+          <t>1-1700170122242</t>
         </is>
       </c>
       <c r="K9" t="inlineStr"/>
@@ -996,12 +996,12 @@
       <c r="M9" t="inlineStr"/>
       <c r="N9" t="inlineStr">
         <is>
-          <t>250019908</t>
+          <t>250018231</t>
         </is>
       </c>
       <c r="O9" t="inlineStr">
         <is>
-          <t>250019908</t>
+          <t>250018231</t>
         </is>
       </c>
       <c r="P9" t="inlineStr"/>
@@ -1016,27 +1016,27 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>11811735665</t>
+          <t>37490124824</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>TIM CONTROLE A PLUS - 31,99</t>
+          <t>CONTROLE A PLUS - SP 24,99</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>31,99</t>
+          <t>24,99</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>38999666812</t>
+          <t>14997254839</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>38991942836</t>
+          <t>14981619124</t>
         </is>
       </c>
       <c r="F10" t="inlineStr"/>
@@ -1044,12 +1044,12 @@
       <c r="H10" t="inlineStr"/>
       <c r="I10" t="inlineStr">
         <is>
-          <t>1-1701318822588</t>
+          <t>1-1699028101154</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>1-1701318822588</t>
+          <t>1-1699028101154</t>
         </is>
       </c>
       <c r="K10" t="inlineStr"/>
@@ -1057,12 +1057,12 @@
       <c r="M10" t="inlineStr"/>
       <c r="N10" t="inlineStr">
         <is>
-          <t>250019539</t>
+          <t>250017314</t>
         </is>
       </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t>250019539</t>
+          <t>250017314</t>
         </is>
       </c>
       <c r="P10" t="inlineStr"/>
@@ -1077,7 +1077,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>65096967700</t>
+          <t>90919564453</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -1092,12 +1092,12 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>21998898866</t>
+          <t>81986866449</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>21982553210</t>
+          <t>81996128392</t>
         </is>
       </c>
       <c r="F11" t="inlineStr"/>
@@ -1105,12 +1105,12 @@
       <c r="H11" t="inlineStr"/>
       <c r="I11" t="inlineStr">
         <is>
-          <t>1-1701290446329</t>
+          <t>1-1698575727635</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>1-1701290446329</t>
+          <t>1-1698575727635</t>
         </is>
       </c>
       <c r="K11" t="inlineStr"/>
@@ -1118,12 +1118,12 @@
       <c r="M11" t="inlineStr"/>
       <c r="N11" t="inlineStr">
         <is>
-          <t>250019485</t>
+          <t>250016952</t>
         </is>
       </c>
       <c r="O11" t="inlineStr">
         <is>
-          <t>250019485</t>
+          <t>250016952</t>
         </is>
       </c>
       <c r="P11" t="inlineStr"/>
@@ -1138,27 +1138,27 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>17498382652</t>
+          <t>59808268668</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>TIM CONTROLE A PLUS - 29,99</t>
+          <t>CONTROLE A PLUS - SP 24,99</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>29,99</t>
+          <t>24,99</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>31987484447</t>
+          <t>34999743173</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>31991144960</t>
+          <t>34991255444</t>
         </is>
       </c>
       <c r="F12" t="inlineStr"/>
@@ -1166,12 +1166,12 @@
       <c r="H12" t="inlineStr"/>
       <c r="I12" t="inlineStr">
         <is>
-          <t>1-1701290444848</t>
+          <t>1-1697841066443</t>
         </is>
       </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>1-1701290444848</t>
+          <t>1-1697841066443</t>
         </is>
       </c>
       <c r="K12" t="inlineStr"/>
@@ -1179,12 +1179,12 @@
       <c r="M12" t="inlineStr"/>
       <c r="N12" t="inlineStr">
         <is>
-          <t>250019490</t>
+          <t>250016265</t>
         </is>
       </c>
       <c r="O12" t="inlineStr">
         <is>
-          <t>250019490</t>
+          <t>250016265</t>
         </is>
       </c>
       <c r="P12" t="inlineStr"/>
@@ -1199,27 +1199,27 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>31280601850</t>
+          <t>04660615600</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>TIM CONTROLE A PLUS - 29,99</t>
+          <t>CONTROLE A PLUS - SP 24,99</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>29,99</t>
+          <t>24,99</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>11972120276</t>
+          <t>38998984148</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>11985584636</t>
+          <t>38991218398</t>
         </is>
       </c>
       <c r="F13" t="inlineStr"/>
@@ -1227,12 +1227,12 @@
       <c r="H13" t="inlineStr"/>
       <c r="I13" t="inlineStr">
         <is>
-          <t>1-1701262473921</t>
+          <t>1-1700001931118</t>
         </is>
       </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>1-1701262473921</t>
+          <t>1-1700001931118</t>
         </is>
       </c>
       <c r="K13" t="inlineStr"/>
@@ -1240,12 +1240,12 @@
       <c r="M13" t="inlineStr"/>
       <c r="N13" t="inlineStr">
         <is>
-          <t>250019433</t>
+          <t>250016070</t>
         </is>
       </c>
       <c r="O13" t="inlineStr">
         <is>
-          <t>250019433</t>
+          <t>250016070</t>
         </is>
       </c>
       <c r="P13" t="inlineStr"/>
@@ -1260,7 +1260,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>28684516672</t>
+          <t>76971023900</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -1275,12 +1275,12 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>35998413419</t>
+          <t>49991415354</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>35991287693</t>
+          <t>49999979360</t>
         </is>
       </c>
       <c r="F14" t="inlineStr"/>
@@ -1288,12 +1288,12 @@
       <c r="H14" t="inlineStr"/>
       <c r="I14" t="inlineStr">
         <is>
-          <t>1-1701298703548</t>
+          <t>1-1697213338435</t>
         </is>
       </c>
       <c r="J14" t="inlineStr">
         <is>
-          <t>1-1701298703548</t>
+          <t>1-1697213338435</t>
         </is>
       </c>
       <c r="K14" t="inlineStr"/>
@@ -1301,12 +1301,12 @@
       <c r="M14" t="inlineStr"/>
       <c r="N14" t="inlineStr">
         <is>
-          <t>250019293</t>
+          <t>250015726</t>
         </is>
       </c>
       <c r="O14" t="inlineStr">
         <is>
-          <t>250019293</t>
+          <t>250015726</t>
         </is>
       </c>
       <c r="P14" t="inlineStr"/>
@@ -1321,27 +1321,27 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>17979850785</t>
+          <t>88184560672</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>TIM CONTROLE A PLUS - 29,99</t>
+          <t>TIM CONTROLE A PLUS - 31,99</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>29,99</t>
+          <t>31,99</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>21995145778</t>
+          <t>31986900068</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>21982768898</t>
+          <t>31991874149</t>
         </is>
       </c>
       <c r="F15" t="inlineStr"/>
@@ -1349,12 +1349,12 @@
       <c r="H15" t="inlineStr"/>
       <c r="I15" t="inlineStr">
         <is>
-          <t>1-1702205491001</t>
+          <t>1-1697190217846</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
         <is>
-          <t>1-1702205491001</t>
+          <t>1-1697190217846</t>
         </is>
       </c>
       <c r="K15" t="inlineStr"/>
@@ -1362,12 +1362,12 @@
       <c r="M15" t="inlineStr"/>
       <c r="N15" t="inlineStr">
         <is>
-          <t>250019221</t>
+          <t>250015710</t>
         </is>
       </c>
       <c r="O15" t="inlineStr">
         <is>
-          <t>250019221</t>
+          <t>250015710</t>
         </is>
       </c>
       <c r="P15" t="inlineStr"/>
@@ -1382,27 +1382,27 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>10841090777</t>
+          <t>38891971839</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>TIM CONTROLE A PLUS - 29,99</t>
+          <t>CONTROLE A PLUS - SP 24,99</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>29,99</t>
+          <t>24,99</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>21993386433</t>
+          <t>13998045270</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>21981924829</t>
+          <t>13981907948</t>
         </is>
       </c>
       <c r="F16" t="inlineStr"/>
@@ -1410,12 +1410,12 @@
       <c r="H16" t="inlineStr"/>
       <c r="I16" t="inlineStr">
         <is>
-          <t>1-1700409431036</t>
+          <t>1-1697147326140</t>
         </is>
       </c>
       <c r="J16" t="inlineStr">
         <is>
-          <t>1-1700409431036</t>
+          <t>1-1697147326140</t>
         </is>
       </c>
       <c r="K16" t="inlineStr"/>
@@ -1423,12 +1423,12 @@
       <c r="M16" t="inlineStr"/>
       <c r="N16" t="inlineStr">
         <is>
-          <t>250018444</t>
+          <t>250015666</t>
         </is>
       </c>
       <c r="O16" t="inlineStr">
         <is>
-          <t>250018444</t>
+          <t>250015666</t>
         </is>
       </c>
       <c r="P16" t="inlineStr"/>
@@ -1443,27 +1443,27 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>41779026838</t>
+          <t>66216664034</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>CONTROLE A PLUS - SP 24,99</t>
+          <t>TIM CONTROLE SMART - DESC 43 - 46,99</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>24,99</t>
+          <t>46,99</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>11916376562</t>
+          <t>54999099995</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>11982502898</t>
+          <t>54981275138</t>
         </is>
       </c>
       <c r="F17" t="inlineStr"/>
@@ -1471,12 +1471,12 @@
       <c r="H17" t="inlineStr"/>
       <c r="I17" t="inlineStr">
         <is>
-          <t>1-1700516997814</t>
+          <t>1-1696625790426</t>
         </is>
       </c>
       <c r="J17" t="inlineStr">
         <is>
-          <t>1-1700516997814</t>
+          <t>1-1696625790426</t>
         </is>
       </c>
       <c r="K17" t="inlineStr"/>
@@ -1484,12 +1484,12 @@
       <c r="M17" t="inlineStr"/>
       <c r="N17" t="inlineStr">
         <is>
-          <t>250018670</t>
+          <t>250015365</t>
         </is>
       </c>
       <c r="O17" t="inlineStr">
         <is>
-          <t>250018670</t>
+          <t>250015365</t>
         </is>
       </c>
       <c r="P17" t="inlineStr"/>
@@ -1504,27 +1504,27 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>34126187804</t>
+          <t>62814354191</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>CONTROLE A PLUS - SP 24,99</t>
+          <t>TIM CONTROLE A PLUS - 29,99</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>24,99</t>
+          <t>29,99</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>19993830911</t>
+          <t>67981018024</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>19981219578</t>
+          <t>67981463441</t>
         </is>
       </c>
       <c r="F18" t="inlineStr"/>
@@ -1532,12 +1532,12 @@
       <c r="H18" t="inlineStr"/>
       <c r="I18" t="inlineStr">
         <is>
-          <t>1-1700329520998</t>
+          <t>1-1696325266270</t>
         </is>
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>1-1700329520998</t>
+          <t>1-1696325266270</t>
         </is>
       </c>
       <c r="K18" t="inlineStr"/>
@@ -1545,12 +1545,12 @@
       <c r="M18" t="inlineStr"/>
       <c r="N18" t="inlineStr">
         <is>
-          <t>250018363</t>
+          <t>250015076</t>
         </is>
       </c>
       <c r="O18" t="inlineStr">
         <is>
-          <t>250018363</t>
+          <t>250015076</t>
         </is>
       </c>
       <c r="P18" t="inlineStr"/>
@@ -1565,7 +1565,7 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>11419169750</t>
+          <t>11099563712</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
@@ -1580,12 +1580,12 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>27998532257</t>
+          <t>21964752532</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>27981244078</t>
+          <t>21982282321</t>
         </is>
       </c>
       <c r="F19" t="inlineStr"/>
@@ -1593,12 +1593,12 @@
       <c r="H19" t="inlineStr"/>
       <c r="I19" t="inlineStr">
         <is>
-          <t>1-1700292263643</t>
+          <t>1-1701016135198</t>
         </is>
       </c>
       <c r="J19" t="inlineStr">
         <is>
-          <t>1-1700292263643</t>
+          <t>1-1701016135198</t>
         </is>
       </c>
       <c r="K19" t="inlineStr"/>
@@ -1606,12 +1606,12 @@
       <c r="M19" t="inlineStr"/>
       <c r="N19" t="inlineStr">
         <is>
-          <t>250018312</t>
+          <t>250014889</t>
         </is>
       </c>
       <c r="O19" t="inlineStr">
         <is>
-          <t>250018312</t>
+          <t>250014889</t>
         </is>
       </c>
       <c r="P19" t="inlineStr"/>
@@ -1626,27 +1626,27 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>36424552634</t>
+          <t>99690012487</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>TIM CONTROLE A PLUS - 31,99</t>
+          <t>TIM CONTROLE A PLUS - 29,99</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>31,99</t>
+          <t>29,99</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>37999748968</t>
+          <t>83993146244</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>37991247780</t>
+          <t>83999869068</t>
         </is>
       </c>
       <c r="F20" t="inlineStr"/>
@@ -1654,12 +1654,12 @@
       <c r="H20" t="inlineStr"/>
       <c r="I20" t="inlineStr">
         <is>
-          <t>1-1700335571847</t>
+          <t>1-1695836175392</t>
         </is>
       </c>
       <c r="J20" t="inlineStr">
         <is>
-          <t>1-1700335571847</t>
+          <t>1-1695836175392</t>
         </is>
       </c>
       <c r="K20" t="inlineStr"/>
@@ -1667,12 +1667,12 @@
       <c r="M20" t="inlineStr"/>
       <c r="N20" t="inlineStr">
         <is>
-          <t>250018415</t>
+          <t>250014820</t>
         </is>
       </c>
       <c r="O20" t="inlineStr">
         <is>
-          <t>250018415</t>
+          <t>250014820</t>
         </is>
       </c>
       <c r="P20" t="inlineStr"/>
@@ -1687,27 +1687,27 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>35226886861</t>
+          <t>96756012134</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>CONTROLE A PLUS - SP 24,99</t>
+          <t>TIM CONTROLE A PLUS - 29,99</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>24,99</t>
+          <t>29,99</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>11910797479</t>
+          <t>62994097709</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>11983954689</t>
+          <t>62984452963</t>
         </is>
       </c>
       <c r="F21" t="inlineStr"/>
@@ -1715,12 +1715,12 @@
       <c r="H21" t="inlineStr"/>
       <c r="I21" t="inlineStr">
         <is>
-          <t>1-1700222301620</t>
+          <t>1-1695324180440</t>
         </is>
       </c>
       <c r="J21" t="inlineStr">
         <is>
-          <t>1-1700222301620</t>
+          <t>1-1695324180440</t>
         </is>
       </c>
       <c r="K21" t="inlineStr"/>
@@ -1728,12 +1728,12 @@
       <c r="M21" t="inlineStr"/>
       <c r="N21" t="inlineStr">
         <is>
-          <t>250018230</t>
+          <t>250014605</t>
         </is>
       </c>
       <c r="O21" t="inlineStr">
         <is>
-          <t>250018230</t>
+          <t>250014605</t>
         </is>
       </c>
       <c r="P21" t="inlineStr"/>
@@ -1748,27 +1748,27 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>79242707287</t>
+          <t>30777739615</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>TIM CONTROLE A PLUS - 29,99</t>
+          <t>TIM CONTROLE A PLUS - 31,99</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>29,99</t>
+          <t>31,99</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>68999495664</t>
+          <t>33984285910</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>68981018609</t>
+          <t>33991486876</t>
         </is>
       </c>
       <c r="F22" t="inlineStr"/>
@@ -1776,12 +1776,12 @@
       <c r="H22" t="inlineStr"/>
       <c r="I22" t="inlineStr">
         <is>
-          <t>1-1700165301441</t>
+          <t>1-1695149109351</t>
         </is>
       </c>
       <c r="J22" t="inlineStr">
         <is>
-          <t>1-1700165301441</t>
+          <t>1-1695149109351</t>
         </is>
       </c>
       <c r="K22" t="inlineStr"/>
@@ -1789,12 +1789,12 @@
       <c r="M22" t="inlineStr"/>
       <c r="N22" t="inlineStr">
         <is>
-          <t>250018159</t>
+          <t>250014570</t>
         </is>
       </c>
       <c r="O22" t="inlineStr">
         <is>
-          <t>250018159</t>
+          <t>250014570</t>
         </is>
       </c>
       <c r="P22" t="inlineStr"/>
@@ -1809,27 +1809,27 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>15731636605</t>
+          <t>36980270893</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>CONTROLE A PLUS - SP 24,99</t>
+          <t>TIM CONTROLE A PLUS - 31,99</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>24,99</t>
+          <t>31,99</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>12988329818</t>
+          <t>17991326935</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>12982946757</t>
+          <t>17981484267</t>
         </is>
       </c>
       <c r="F23" t="inlineStr"/>
@@ -1837,12 +1837,12 @@
       <c r="H23" t="inlineStr"/>
       <c r="I23" t="inlineStr">
         <is>
-          <t>1-1700166746401</t>
+          <t>1-1695162177188</t>
         </is>
       </c>
       <c r="J23" t="inlineStr">
         <is>
-          <t>1-1700166746401</t>
+          <t>1-1695162177188</t>
         </is>
       </c>
       <c r="K23" t="inlineStr"/>
@@ -1850,12 +1850,12 @@
       <c r="M23" t="inlineStr"/>
       <c r="N23" t="inlineStr">
         <is>
-          <t>250018171</t>
+          <t>250014559</t>
         </is>
       </c>
       <c r="O23" t="inlineStr">
         <is>
-          <t>250018171</t>
+          <t>250014559</t>
         </is>
       </c>
       <c r="P23" t="inlineStr"/>
@@ -1870,27 +1870,27 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>50849964849</t>
+          <t>46980601091</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>CONTROLE A PLUS - SP 24,99</t>
+          <t>TIM CONTROLE A PLUS - 29,99</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>24,99</t>
+          <t>29,99</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>11942301412</t>
+          <t>99984747337</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>11983958201</t>
+          <t>99981995421</t>
         </is>
       </c>
       <c r="F24" t="inlineStr"/>
@@ -1898,12 +1898,12 @@
       <c r="H24" t="inlineStr"/>
       <c r="I24" t="inlineStr">
         <is>
-          <t>1-1700290243600</t>
+          <t>1-1693408713994</t>
         </is>
       </c>
       <c r="J24" t="inlineStr">
         <is>
-          <t>1-1700290243600</t>
+          <t>1-1693408713994</t>
         </is>
       </c>
       <c r="K24" t="inlineStr"/>
@@ -1911,12 +1911,12 @@
       <c r="M24" t="inlineStr"/>
       <c r="N24" t="inlineStr">
         <is>
-          <t>250018145</t>
+          <t>250014036</t>
         </is>
       </c>
       <c r="O24" t="inlineStr">
         <is>
-          <t>250018145</t>
+          <t>250014036</t>
         </is>
       </c>
       <c r="P24" t="inlineStr"/>
@@ -1931,7 +1931,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>60265804094</t>
+          <t>40564356859</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -1946,12 +1946,12 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>51997675242</t>
+          <t>13974178341</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>51981753434</t>
+          <t>13981714602</t>
         </is>
       </c>
       <c r="F25" t="inlineStr"/>
@@ -1959,12 +1959,12 @@
       <c r="H25" t="inlineStr"/>
       <c r="I25" t="inlineStr">
         <is>
-          <t>1-1699882364677</t>
+          <t>1-1692260914320</t>
         </is>
       </c>
       <c r="J25" t="inlineStr">
         <is>
-          <t>1-1699882364677</t>
+          <t>1-1692260914320</t>
         </is>
       </c>
       <c r="K25" t="inlineStr"/>
@@ -1972,12 +1972,12 @@
       <c r="M25" t="inlineStr"/>
       <c r="N25" t="inlineStr">
         <is>
-          <t>250018025</t>
+          <t>250013865</t>
         </is>
       </c>
       <c r="O25" t="inlineStr">
         <is>
-          <t>250018025</t>
+          <t>250013865</t>
         </is>
       </c>
       <c r="P25" t="inlineStr"/>
@@ -1992,27 +1992,27 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>17353446803</t>
+          <t>21693258838</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>TIM CONTROLE A PLUS - 29,99</t>
+          <t>TIM CONTROLE SMART - DESC 43 - 46,99</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>29,99</t>
+          <t>46,99</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>11968667516</t>
+          <t>15988190123</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>11970225621</t>
+          <t>15981808632</t>
         </is>
       </c>
       <c r="F26" t="inlineStr"/>
@@ -2020,12 +2020,12 @@
       <c r="H26" t="inlineStr"/>
       <c r="I26" t="inlineStr">
         <is>
-          <t>1-1702616327192</t>
+          <t>1-1689396586860</t>
         </is>
       </c>
       <c r="J26" t="inlineStr">
         <is>
-          <t>1-1702616327192</t>
+          <t>1-1689396586860</t>
         </is>
       </c>
       <c r="K26" t="inlineStr"/>
@@ -2033,12 +2033,12 @@
       <c r="M26" t="inlineStr"/>
       <c r="N26" t="inlineStr">
         <is>
-          <t>250017944</t>
+          <t>250013324</t>
         </is>
       </c>
       <c r="O26" t="inlineStr">
         <is>
-          <t>250017944</t>
+          <t>250013324</t>
         </is>
       </c>
       <c r="P26" t="inlineStr"/>
@@ -2053,27 +2053,27 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>33814641833</t>
+          <t>16715651850</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>TIM CONTROLE A PLUS - 29,99</t>
+          <t>TIM CONTROLE A PLUS - 31,99</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>29,99</t>
+          <t>31,99</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>92994329660</t>
+          <t>17991898544</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>92981144376</t>
+          <t>17981325353</t>
         </is>
       </c>
       <c r="F27" t="inlineStr"/>
@@ -2081,12 +2081,12 @@
       <c r="H27" t="inlineStr"/>
       <c r="I27" t="inlineStr">
         <is>
-          <t>1-1701292678994</t>
+          <t>1-1689425557597</t>
         </is>
       </c>
       <c r="J27" t="inlineStr">
         <is>
-          <t>1-1701292678994</t>
+          <t>1-1689425557597</t>
         </is>
       </c>
       <c r="K27" t="inlineStr"/>
@@ -2094,12 +2094,12 @@
       <c r="M27" t="inlineStr"/>
       <c r="N27" t="inlineStr">
         <is>
-          <t>250017476</t>
+          <t>250013307</t>
         </is>
       </c>
       <c r="O27" t="inlineStr">
         <is>
-          <t>250017476</t>
+          <t>250013307</t>
         </is>
       </c>
       <c r="P27" t="inlineStr"/>
@@ -2114,27 +2114,27 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>11300796782</t>
+          <t>27616061672</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>TIM CONTROLE A PLUS - 29,99</t>
+          <t>TIM CONTROLE A PLUS - 31,99</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>29,99</t>
+          <t>31,99</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>21997637433</t>
+          <t>37999295606</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>21982020627</t>
+          <t>37991408075</t>
         </is>
       </c>
       <c r="F28" t="inlineStr"/>
@@ -2142,12 +2142,12 @@
       <c r="H28" t="inlineStr"/>
       <c r="I28" t="inlineStr">
         <is>
-          <t>1-1699325652122</t>
+          <t>1-1689195359331</t>
         </is>
       </c>
       <c r="J28" t="inlineStr">
         <is>
-          <t>1-1699325652122</t>
+          <t>1-1689195359331</t>
         </is>
       </c>
       <c r="K28" t="inlineStr"/>
@@ -2155,12 +2155,12 @@
       <c r="M28" t="inlineStr"/>
       <c r="N28" t="inlineStr">
         <is>
-          <t>250017471</t>
+          <t>250013175</t>
         </is>
       </c>
       <c r="O28" t="inlineStr">
         <is>
-          <t>250017471</t>
+          <t>250013175</t>
         </is>
       </c>
       <c r="P28" t="inlineStr"/>
@@ -2175,27 +2175,27 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>37490124824</t>
+          <t>12491153882</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>CONTROLE A PLUS - SP 24,99</t>
+          <t>TIM CONTROLE A PLUS - 31,99</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>24,99</t>
+          <t>31,99</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>14997254839</t>
+          <t>17997432898</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>14981619124</t>
+          <t>17981315240</t>
         </is>
       </c>
       <c r="F29" t="inlineStr"/>
@@ -2203,12 +2203,12 @@
       <c r="H29" t="inlineStr"/>
       <c r="I29" t="inlineStr">
         <is>
-          <t>1-1699028101154</t>
+          <t>1-1689022733709</t>
         </is>
       </c>
       <c r="J29" t="inlineStr">
         <is>
-          <t>1-1699028101154</t>
+          <t>1-1689022733709</t>
         </is>
       </c>
       <c r="K29" t="inlineStr"/>
@@ -2216,12 +2216,12 @@
       <c r="M29" t="inlineStr"/>
       <c r="N29" t="inlineStr">
         <is>
-          <t>250017314</t>
+          <t>250012941</t>
         </is>
       </c>
       <c r="O29" t="inlineStr">
         <is>
-          <t>250017314</t>
+          <t>250012941</t>
         </is>
       </c>
       <c r="P29" t="inlineStr"/>
@@ -2236,27 +2236,27 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>90919564453</t>
+          <t>21997111888</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>TIM CONTROLE A PLUS - 29,99</t>
+          <t>TIM CONTROLE A PLUS - 31,99</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>29,99</t>
+          <t>31,99</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>81986866449</t>
+          <t>11991202951</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>81996128392</t>
+          <t>11983422357</t>
         </is>
       </c>
       <c r="F30" t="inlineStr"/>
@@ -2264,12 +2264,12 @@
       <c r="H30" t="inlineStr"/>
       <c r="I30" t="inlineStr">
         <is>
-          <t>1-1698575727635</t>
+          <t>1-1689055400944</t>
         </is>
       </c>
       <c r="J30" t="inlineStr">
         <is>
-          <t>1-1698575727635</t>
+          <t>1-1689055400944</t>
         </is>
       </c>
       <c r="K30" t="inlineStr"/>
@@ -2277,12 +2277,12 @@
       <c r="M30" t="inlineStr"/>
       <c r="N30" t="inlineStr">
         <is>
-          <t>250016952</t>
+          <t>250013065</t>
         </is>
       </c>
       <c r="O30" t="inlineStr">
         <is>
-          <t>250016952</t>
+          <t>250013065</t>
         </is>
       </c>
       <c r="P30" t="inlineStr"/>
@@ -2297,27 +2297,27 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>90980131553</t>
+          <t>59073810604</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>TIM CONTROLE A PLUS - 29,99</t>
+          <t>TIM CONTROLE A PLUS - 31,99</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>29,99</t>
+          <t>31,99</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>77998706726</t>
+          <t>37999957772</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>77991576212</t>
+          <t>37991315436</t>
         </is>
       </c>
       <c r="F31" t="inlineStr"/>
@@ -2325,12 +2325,12 @@
       <c r="H31" t="inlineStr"/>
       <c r="I31" t="inlineStr">
         <is>
-          <t>1-1698450502840</t>
+          <t>1-1688875815921</t>
         </is>
       </c>
       <c r="J31" t="inlineStr">
         <is>
-          <t>1-1698450502840</t>
+          <t>1-1688875815921</t>
         </is>
       </c>
       <c r="K31" t="inlineStr"/>
@@ -2338,12 +2338,12 @@
       <c r="M31" t="inlineStr"/>
       <c r="N31" t="inlineStr">
         <is>
-          <t>250016822</t>
+          <t>250012786</t>
         </is>
       </c>
       <c r="O31" t="inlineStr">
         <is>
-          <t>250016822</t>
+          <t>250012786</t>
         </is>
       </c>
       <c r="P31" t="inlineStr"/>
@@ -2358,27 +2358,27 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>05083245647</t>
+          <t>32805448820</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>TIM CONTROLE A PLUS - 29,99</t>
+          <t>TIM CONTROLE A PLUS - 31,99</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>29,99</t>
+          <t>31,99</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>37984005838</t>
+          <t>11971591302</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>37991145411</t>
+          <t>11982046106</t>
         </is>
       </c>
       <c r="F32" t="inlineStr"/>
@@ -2386,12 +2386,12 @@
       <c r="H32" t="inlineStr"/>
       <c r="I32" t="inlineStr">
         <is>
-          <t>1-1698176147735</t>
+          <t>1-1691788348780</t>
         </is>
       </c>
       <c r="J32" t="inlineStr">
         <is>
-          <t>1-1698176147735</t>
+          <t>1-1691788348780</t>
         </is>
       </c>
       <c r="K32" t="inlineStr"/>
@@ -2399,12 +2399,12 @@
       <c r="M32" t="inlineStr"/>
       <c r="N32" t="inlineStr">
         <is>
-          <t>250016547</t>
+          <t>250012470</t>
         </is>
       </c>
       <c r="O32" t="inlineStr">
         <is>
-          <t>250016547</t>
+          <t>250012470</t>
         </is>
       </c>
       <c r="P32" t="inlineStr"/>
@@ -2419,7 +2419,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>36180343349</t>
+          <t>32540523153</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -2434,12 +2434,12 @@
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>86994354070</t>
+          <t>67996548054</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>86999392671</t>
+          <t>67981710181</t>
         </is>
       </c>
       <c r="F33" t="inlineStr"/>
@@ -2447,12 +2447,12 @@
       <c r="H33" t="inlineStr"/>
       <c r="I33" t="inlineStr">
         <is>
-          <t>1-1700040675082</t>
+          <t>1-1688368309027</t>
         </is>
       </c>
       <c r="J33" t="inlineStr">
         <is>
-          <t>1-1700040675082</t>
+          <t>1-1688368309027</t>
         </is>
       </c>
       <c r="K33" t="inlineStr"/>
@@ -2460,12 +2460,12 @@
       <c r="M33" t="inlineStr"/>
       <c r="N33" t="inlineStr">
         <is>
-          <t>250016413</t>
+          <t>250012214</t>
         </is>
       </c>
       <c r="O33" t="inlineStr">
         <is>
-          <t>250016413</t>
+          <t>250012214</t>
         </is>
       </c>
       <c r="P33" t="inlineStr"/>
@@ -2480,27 +2480,27 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>39624123870</t>
+          <t>35152513838</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>CONTROLE A PLUS - SP 24,99</t>
+          <t>TIM CONTROLE A PLUS - 31,99</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>24,99</t>
+          <t>31,99</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>12996451969</t>
+          <t>18998113387</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>12982909107</t>
+          <t>18981793506</t>
         </is>
       </c>
       <c r="F34" t="inlineStr"/>
@@ -2508,12 +2508,12 @@
       <c r="H34" t="inlineStr"/>
       <c r="I34" t="inlineStr">
         <is>
-          <t>1-1697998309349</t>
+          <t>1-1688335913716</t>
         </is>
       </c>
       <c r="J34" t="inlineStr">
         <is>
-          <t>1-1697998309349</t>
+          <t>1-1688335913716</t>
         </is>
       </c>
       <c r="K34" t="inlineStr"/>
@@ -2521,12 +2521,12 @@
       <c r="M34" t="inlineStr"/>
       <c r="N34" t="inlineStr">
         <is>
-          <t>250016350</t>
+          <t>250012155</t>
         </is>
       </c>
       <c r="O34" t="inlineStr">
         <is>
-          <t>250016350</t>
+          <t>250012155</t>
         </is>
       </c>
       <c r="P34" t="inlineStr"/>
@@ -2541,27 +2541,27 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>59808268668</t>
+          <t>31723846830</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>CONTROLE A PLUS - SP 24,99</t>
+          <t>TIM CONTROLE A PLUS - 29,99</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>24,99</t>
+          <t>29,99</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>34999743173</t>
+          <t>73999443265</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>34991255444</t>
+          <t>73988248564</t>
         </is>
       </c>
       <c r="F35" t="inlineStr"/>
@@ -2569,12 +2569,12 @@
       <c r="H35" t="inlineStr"/>
       <c r="I35" t="inlineStr">
         <is>
-          <t>1-1697841066443</t>
+          <t>1-1700577967983</t>
         </is>
       </c>
       <c r="J35" t="inlineStr">
         <is>
-          <t>1-1697841066443</t>
+          <t>1-1700577967983</t>
         </is>
       </c>
       <c r="K35" t="inlineStr"/>
@@ -2582,12 +2582,12 @@
       <c r="M35" t="inlineStr"/>
       <c r="N35" t="inlineStr">
         <is>
-          <t>250016265</t>
+          <t>250012231</t>
         </is>
       </c>
       <c r="O35" t="inlineStr">
         <is>
-          <t>250016265</t>
+          <t>250012231</t>
         </is>
       </c>
       <c r="P35" t="inlineStr"/>
@@ -2602,27 +2602,27 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>10140528660</t>
+          <t>51565170482</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>TIM CONTROLE A PLUS - 31,99</t>
+          <t>TIM CONTROLE A PLUS - 29,99</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>31,99</t>
+          <t>29,99</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>35991000892</t>
+          <t>81999106660</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>35991263861</t>
+          <t>81999057235</t>
         </is>
       </c>
       <c r="F36" t="inlineStr"/>
@@ -2630,12 +2630,12 @@
       <c r="H36" t="inlineStr"/>
       <c r="I36" t="inlineStr">
         <is>
-          <t>1-1697727605549</t>
+          <t>1-1688259134952</t>
         </is>
       </c>
       <c r="J36" t="inlineStr">
         <is>
-          <t>1-1697727605549</t>
+          <t>1-1688259134952</t>
         </is>
       </c>
       <c r="K36" t="inlineStr"/>
@@ -2643,12 +2643,12 @@
       <c r="M36" t="inlineStr"/>
       <c r="N36" t="inlineStr">
         <is>
-          <t>250016185</t>
+          <t>250012145</t>
         </is>
       </c>
       <c r="O36" t="inlineStr">
         <is>
-          <t>250016185</t>
+          <t>250012145</t>
         </is>
       </c>
       <c r="P36" t="inlineStr"/>
@@ -2663,7 +2663,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>02456945018</t>
+          <t>68436637372</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -2678,12 +2678,12 @@
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>55996481377</t>
+          <t>11992139465</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>55981392355</t>
+          <t>11984612562</t>
         </is>
       </c>
       <c r="F37" t="inlineStr"/>
@@ -2691,12 +2691,12 @@
       <c r="H37" t="inlineStr"/>
       <c r="I37" t="inlineStr">
         <is>
-          <t>1-1697668179573</t>
+          <t>1-1688060258052</t>
         </is>
       </c>
       <c r="J37" t="inlineStr">
         <is>
-          <t>1-1697668179573</t>
+          <t>1-1688060258052</t>
         </is>
       </c>
       <c r="K37" t="inlineStr"/>
@@ -2704,12 +2704,12 @@
       <c r="M37" t="inlineStr"/>
       <c r="N37" t="inlineStr">
         <is>
-          <t>250016075</t>
+          <t>250011869</t>
         </is>
       </c>
       <c r="O37" t="inlineStr">
         <is>
-          <t>250016075</t>
+          <t>250011869</t>
         </is>
       </c>
       <c r="P37" t="inlineStr"/>
@@ -2724,27 +2724,27 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>04660615600</t>
+          <t>10370108680</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>CONTROLE A PLUS - SP 24,99</t>
+          <t>TIM CONTROLE A PLUS - 31,99</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>24,99</t>
+          <t>31,99</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>38998984148</t>
+          <t>33999370050</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>38991218398</t>
+          <t>33991718645</t>
         </is>
       </c>
       <c r="F38" t="inlineStr"/>
@@ -2752,12 +2752,12 @@
       <c r="H38" t="inlineStr"/>
       <c r="I38" t="inlineStr">
         <is>
-          <t>1-1700001931118</t>
+          <t>1-1687489415039</t>
         </is>
       </c>
       <c r="J38" t="inlineStr">
         <is>
-          <t>1-1700001931118</t>
+          <t>1-1687489415039</t>
         </is>
       </c>
       <c r="K38" t="inlineStr"/>
@@ -2765,12 +2765,12 @@
       <c r="M38" t="inlineStr"/>
       <c r="N38" t="inlineStr">
         <is>
-          <t>250016070</t>
+          <t>250011290</t>
         </is>
       </c>
       <c r="O38" t="inlineStr">
         <is>
-          <t>250016070</t>
+          <t>250011290</t>
         </is>
       </c>
       <c r="P38" t="inlineStr"/>
@@ -2785,27 +2785,27 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>73565334134</t>
+          <t>42319361880</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>TIM CONTROLE A PLUS - 29,99</t>
+          <t>TIM CONTROLE A PLUS - 31,99</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>29,99</t>
+          <t>31,99</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>61995818953</t>
+          <t>18996536961</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>61981730827</t>
+          <t>18981928980</t>
         </is>
       </c>
       <c r="F39" t="inlineStr"/>
@@ -2813,12 +2813,12 @@
       <c r="H39" t="inlineStr"/>
       <c r="I39" t="inlineStr">
         <is>
-          <t>1-1697260088766</t>
+          <t>1-1687472463902</t>
         </is>
       </c>
       <c r="J39" t="inlineStr">
         <is>
-          <t>1-1697260088766</t>
+          <t>1-1687472463902</t>
         </is>
       </c>
       <c r="K39" t="inlineStr"/>
@@ -2826,12 +2826,12 @@
       <c r="M39" t="inlineStr"/>
       <c r="N39" t="inlineStr">
         <is>
-          <t>250015739</t>
+          <t>250011277</t>
         </is>
       </c>
       <c r="O39" t="inlineStr">
         <is>
-          <t>250015739</t>
+          <t>250011277</t>
         </is>
       </c>
       <c r="P39" t="inlineStr"/>
@@ -2846,27 +2846,27 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>05064621450</t>
+          <t>10294115650</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>TIM CONTROLE A PLUS - 29,99</t>
+          <t>TIM CONTROLE A PLUS - 31,99</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>29,99</t>
+          <t>31,99</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>81993951498</t>
+          <t>33999820674</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>81999657872</t>
+          <t>33991984404</t>
         </is>
       </c>
       <c r="F40" t="inlineStr"/>
@@ -2874,12 +2874,12 @@
       <c r="H40" t="inlineStr"/>
       <c r="I40" t="inlineStr">
         <is>
-          <t>1-1697307322532</t>
+          <t>1-1687489795621</t>
         </is>
       </c>
       <c r="J40" t="inlineStr">
         <is>
-          <t>1-1697307322532</t>
+          <t>1-1687489795621</t>
         </is>
       </c>
       <c r="K40" t="inlineStr"/>
@@ -2887,12 +2887,12 @@
       <c r="M40" t="inlineStr"/>
       <c r="N40" t="inlineStr">
         <is>
-          <t>250015796</t>
+          <t>250011297</t>
         </is>
       </c>
       <c r="O40" t="inlineStr">
         <is>
-          <t>250015796</t>
+          <t>250011297</t>
         </is>
       </c>
       <c r="P40" t="inlineStr"/>
@@ -2907,7 +2907,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>84034980559</t>
+          <t>10786518766</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -2922,12 +2922,12 @@
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>71982158094</t>
+          <t>21978878310</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>71993536534</t>
+          <t>21981581449</t>
         </is>
       </c>
       <c r="F41" t="inlineStr"/>
@@ -2935,12 +2935,12 @@
       <c r="H41" t="inlineStr"/>
       <c r="I41" t="inlineStr">
         <is>
-          <t>1-1697263981433</t>
+          <t>1-1687462499765</t>
         </is>
       </c>
       <c r="J41" t="inlineStr">
         <is>
-          <t>1-1697263981433</t>
+          <t>1-1687462499765</t>
         </is>
       </c>
       <c r="K41" t="inlineStr"/>
@@ -2948,12 +2948,12 @@
       <c r="M41" t="inlineStr"/>
       <c r="N41" t="inlineStr">
         <is>
-          <t>250015738</t>
+          <t>250011247</t>
         </is>
       </c>
       <c r="O41" t="inlineStr">
         <is>
-          <t>250015738</t>
+          <t>250011247</t>
         </is>
       </c>
       <c r="P41" t="inlineStr"/>
@@ -2968,27 +2968,27 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>76971023900</t>
+          <t>73590991453</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>TIM CONTROLE A PLUS - 31,99</t>
+          <t>TIM CONTROLE A PLUS - 29,99</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>31,99</t>
+          <t>29,99</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>49991415354</t>
+          <t>81983850056</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>49999979360</t>
+          <t>81999076032</t>
         </is>
       </c>
       <c r="F42" t="inlineStr"/>
@@ -2996,12 +2996,12 @@
       <c r="H42" t="inlineStr"/>
       <c r="I42" t="inlineStr">
         <is>
-          <t>1-1697213338435</t>
+          <t>1-1687544864575</t>
         </is>
       </c>
       <c r="J42" t="inlineStr">
         <is>
-          <t>1-1697213338435</t>
+          <t>1-1687544864575</t>
         </is>
       </c>
       <c r="K42" t="inlineStr"/>
@@ -3009,12 +3009,12 @@
       <c r="M42" t="inlineStr"/>
       <c r="N42" t="inlineStr">
         <is>
-          <t>250015726</t>
+          <t>250011262</t>
         </is>
       </c>
       <c r="O42" t="inlineStr">
         <is>
-          <t>250015726</t>
+          <t>250011262</t>
         </is>
       </c>
       <c r="P42" t="inlineStr"/>
@@ -3029,27 +3029,27 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>88184560672</t>
+          <t>70246883197</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>TIM CONTROLE A PLUS - 31,99</t>
+          <t>TIM CONTROLE A PLUS - 29,99</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>31,99</t>
+          <t>29,99</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>31986900068</t>
+          <t>64935003714</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>31991874149</t>
+          <t>64981469118</t>
         </is>
       </c>
       <c r="F43" t="inlineStr"/>
@@ -3057,12 +3057,12 @@
       <c r="H43" t="inlineStr"/>
       <c r="I43" t="inlineStr">
         <is>
-          <t>1-1697190217846</t>
+          <t>1-1687305654949</t>
         </is>
       </c>
       <c r="J43" t="inlineStr">
         <is>
-          <t>1-1697190217846</t>
+          <t>1-1687305654949</t>
         </is>
       </c>
       <c r="K43" t="inlineStr"/>
@@ -3070,12 +3070,12 @@
       <c r="M43" t="inlineStr"/>
       <c r="N43" t="inlineStr">
         <is>
-          <t>250015710</t>
+          <t>250011070</t>
         </is>
       </c>
       <c r="O43" t="inlineStr">
         <is>
-          <t>250015710</t>
+          <t>250011070</t>
         </is>
       </c>
       <c r="P43" t="inlineStr"/>
@@ -3090,27 +3090,27 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>38891971839</t>
+          <t>26633304854</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>CONTROLE A PLUS - SP 24,99</t>
+          <t>TIM CONTROLE A PLUS - 31,99</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>24,99</t>
+          <t>31,99</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>13998045270</t>
+          <t>14988069168</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>13981907948</t>
+          <t>14981565025</t>
         </is>
       </c>
       <c r="F44" t="inlineStr"/>
@@ -3118,12 +3118,12 @@
       <c r="H44" t="inlineStr"/>
       <c r="I44" t="inlineStr">
         <is>
-          <t>1-1697147326140</t>
+          <t>1-1687030402589</t>
         </is>
       </c>
       <c r="J44" t="inlineStr">
         <is>
-          <t>1-1697147326140</t>
+          <t>1-1687030402589</t>
         </is>
       </c>
       <c r="K44" t="inlineStr"/>
@@ -3131,12 +3131,12 @@
       <c r="M44" t="inlineStr"/>
       <c r="N44" t="inlineStr">
         <is>
-          <t>250015666</t>
+          <t>250010697</t>
         </is>
       </c>
       <c r="O44" t="inlineStr">
         <is>
-          <t>250015666</t>
+          <t>250010697</t>
         </is>
       </c>
       <c r="P44" t="inlineStr"/>
@@ -3151,27 +3151,27 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>12747532607</t>
+          <t>14976558703</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>TIM CONTROLE A PLUS - 31,99</t>
+          <t>TIM CONTROLE A PLUS - 29,99</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>31,99</t>
+          <t>29,99</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>38984221303</t>
+          <t>21975427182</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>38991931785</t>
+          <t>21989743509</t>
         </is>
       </c>
       <c r="F45" t="inlineStr"/>
@@ -3179,12 +3179,12 @@
       <c r="H45" t="inlineStr"/>
       <c r="I45" t="inlineStr">
         <is>
-          <t>1-1696689313059</t>
+          <t>1-1687095672007</t>
         </is>
       </c>
       <c r="J45" t="inlineStr">
         <is>
-          <t>1-1696689313059</t>
+          <t>1-1687095672007</t>
         </is>
       </c>
       <c r="K45" t="inlineStr"/>
@@ -3192,12 +3192,12 @@
       <c r="M45" t="inlineStr"/>
       <c r="N45" t="inlineStr">
         <is>
-          <t>250015422</t>
+          <t>250010814</t>
         </is>
       </c>
       <c r="O45" t="inlineStr">
         <is>
-          <t>250015422</t>
+          <t>250010814</t>
         </is>
       </c>
       <c r="P45" t="inlineStr"/>
@@ -3212,27 +3212,27 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>66216664034</t>
+          <t>31792839472</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>TIM CONTROLE SMART - DESC 43 - 46,99</t>
+          <t>TIM CONTROLE A PLUS - 29,99</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>46,99</t>
+          <t>29,99</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>54999099995</t>
+          <t>81992850532</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>54981275138</t>
+          <t>81999087618</t>
         </is>
       </c>
       <c r="F46" t="inlineStr"/>
@@ -3240,12 +3240,12 @@
       <c r="H46" t="inlineStr"/>
       <c r="I46" t="inlineStr">
         <is>
-          <t>1-1696625790426</t>
+          <t>1-1686873983402</t>
         </is>
       </c>
       <c r="J46" t="inlineStr">
         <is>
-          <t>1-1696625790426</t>
+          <t>1-1686873983402</t>
         </is>
       </c>
       <c r="K46" t="inlineStr"/>
@@ -3253,12 +3253,12 @@
       <c r="M46" t="inlineStr"/>
       <c r="N46" t="inlineStr">
         <is>
-          <t>250015365</t>
+          <t>250010607</t>
         </is>
       </c>
       <c r="O46" t="inlineStr">
         <is>
-          <t>250015365</t>
+          <t>250010607</t>
         </is>
       </c>
       <c r="P46" t="inlineStr"/>
@@ -3273,27 +3273,27 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>71234055953</t>
+          <t>60348852134</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>TIM CONTROLE A PLUS - 31,99</t>
+          <t>TIM CONTROLE A PLUS - 29,99</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>31,99</t>
+          <t>29,99</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>47996574350</t>
+          <t>61991343196</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>47999949376</t>
+          <t>61981547643</t>
         </is>
       </c>
       <c r="F47" t="inlineStr"/>
@@ -3301,12 +3301,12 @@
       <c r="H47" t="inlineStr"/>
       <c r="I47" t="inlineStr">
         <is>
-          <t>1-1696460415442</t>
+          <t>1-1686595896759</t>
         </is>
       </c>
       <c r="J47" t="inlineStr">
         <is>
-          <t>1-1696460415442</t>
+          <t>1-1686595896759</t>
         </is>
       </c>
       <c r="K47" t="inlineStr"/>
@@ -3314,12 +3314,12 @@
       <c r="M47" t="inlineStr"/>
       <c r="N47" t="inlineStr">
         <is>
-          <t>250015195</t>
+          <t>250010183</t>
         </is>
       </c>
       <c r="O47" t="inlineStr">
         <is>
-          <t>250015195</t>
+          <t>250010183</t>
         </is>
       </c>
       <c r="P47" t="inlineStr"/>
@@ -3334,27 +3334,27 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>62814354191</t>
+          <t>30051772892</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>TIM CONTROLE A PLUS - 29,99</t>
+          <t>TIM CONTROLE A PLUS - 31,99</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>29,99</t>
+          <t>31,99</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>67981018024</t>
+          <t>12996783554</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
         <is>
-          <t>67981463441</t>
+          <t>12982038946</t>
         </is>
       </c>
       <c r="F48" t="inlineStr"/>
@@ -3362,12 +3362,12 @@
       <c r="H48" t="inlineStr"/>
       <c r="I48" t="inlineStr">
         <is>
-          <t>1-1696325266270</t>
+          <t>1-1686658178501</t>
         </is>
       </c>
       <c r="J48" t="inlineStr">
         <is>
-          <t>1-1696325266270</t>
+          <t>1-1686658178501</t>
         </is>
       </c>
       <c r="K48" t="inlineStr"/>
@@ -3375,12 +3375,12 @@
       <c r="M48" t="inlineStr"/>
       <c r="N48" t="inlineStr">
         <is>
-          <t>250015076</t>
+          <t>250010294</t>
         </is>
       </c>
       <c r="O48" t="inlineStr">
         <is>
-          <t>250015076</t>
+          <t>250010294</t>
         </is>
       </c>
       <c r="P48" t="inlineStr"/>
@@ -3395,7 +3395,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>75627752653</t>
+          <t>48418203889</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
@@ -3410,12 +3410,12 @@
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>34998330127</t>
+          <t>13974227853</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>34991265925</t>
+          <t>13981918238</t>
         </is>
       </c>
       <c r="F49" t="inlineStr"/>
@@ -3423,12 +3423,12 @@
       <c r="H49" t="inlineStr"/>
       <c r="I49" t="inlineStr">
         <is>
-          <t>1-1696056167109</t>
+          <t>1-1694249709946</t>
         </is>
       </c>
       <c r="J49" t="inlineStr">
         <is>
-          <t>1-1696056167109</t>
+          <t>1-1694249709946</t>
         </is>
       </c>
       <c r="K49" t="inlineStr"/>
@@ -3436,12 +3436,12 @@
       <c r="M49" t="inlineStr"/>
       <c r="N49" t="inlineStr">
         <is>
-          <t>250014890</t>
+          <t>250010311</t>
         </is>
       </c>
       <c r="O49" t="inlineStr">
         <is>
-          <t>250014890</t>
+          <t>250010311</t>
         </is>
       </c>
       <c r="P49" t="inlineStr"/>
@@ -3456,27 +3456,27 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>76795632768</t>
+          <t>35603189800</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>TIM CONTROLE A PLUS - 29,99</t>
+          <t>TIM CONTROLE A PLUS - 31,99</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>29,99</t>
+          <t>31,99</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>22999335554</t>
+          <t>17991659107</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>22988253313</t>
+          <t>17981214232</t>
         </is>
       </c>
       <c r="F50" t="inlineStr"/>
@@ -3484,12 +3484,12 @@
       <c r="H50" t="inlineStr"/>
       <c r="I50" t="inlineStr">
         <is>
-          <t>1-1696084609673</t>
+          <t>1-1686395125746</t>
         </is>
       </c>
       <c r="J50" t="inlineStr">
         <is>
-          <t>1-1696084609673</t>
+          <t>1-1686395125746</t>
         </is>
       </c>
       <c r="K50" t="inlineStr"/>
@@ -3497,12 +3497,12 @@
       <c r="M50" t="inlineStr"/>
       <c r="N50" t="inlineStr">
         <is>
-          <t>250014925</t>
+          <t>250010118</t>
         </is>
       </c>
       <c r="O50" t="inlineStr">
         <is>
-          <t>250014925</t>
+          <t>250010118</t>
         </is>
       </c>
       <c r="P50" t="inlineStr"/>
@@ -3517,27 +3517,27 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>11099563712</t>
+          <t>11198198656</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>TIM CONTROLE A PLUS - 29,99</t>
+          <t>TIM CONTROLE A PLUS - 31,99</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>29,99</t>
+          <t>31,99</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>21964752532</t>
+          <t>31995828395</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>21982282321</t>
+          <t>31991281302</t>
         </is>
       </c>
       <c r="F51" t="inlineStr"/>
@@ -3545,12 +3545,12 @@
       <c r="H51" t="inlineStr"/>
       <c r="I51" t="inlineStr">
         <is>
-          <t>1-1701016135198</t>
+          <t>1-1686087894828</t>
         </is>
       </c>
       <c r="J51" t="inlineStr">
         <is>
-          <t>1-1701016135198</t>
+          <t>1-1686087894828</t>
         </is>
       </c>
       <c r="K51" t="inlineStr"/>
@@ -3558,12 +3558,12 @@
       <c r="M51" t="inlineStr"/>
       <c r="N51" t="inlineStr">
         <is>
-          <t>250014889</t>
+          <t>250009762</t>
         </is>
       </c>
       <c r="O51" t="inlineStr">
         <is>
-          <t>250014889</t>
+          <t>250009762</t>
         </is>
       </c>
       <c r="P51" t="inlineStr"/>
@@ -3578,7 +3578,7 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>99690012487</t>
+          <t>12649725710</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
@@ -3593,12 +3593,12 @@
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>83993146244</t>
+          <t>21968151982</t>
         </is>
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>83999869068</t>
+          <t>21983381274</t>
         </is>
       </c>
       <c r="F52" t="inlineStr"/>
@@ -3606,12 +3606,12 @@
       <c r="H52" t="inlineStr"/>
       <c r="I52" t="inlineStr">
         <is>
-          <t>1-1695836175392</t>
+          <t>1-1685774658131</t>
         </is>
       </c>
       <c r="J52" t="inlineStr">
         <is>
-          <t>1-1695836175392</t>
+          <t>1-1685774658131</t>
         </is>
       </c>
       <c r="K52" t="inlineStr"/>
@@ -3619,12 +3619,12 @@
       <c r="M52" t="inlineStr"/>
       <c r="N52" t="inlineStr">
         <is>
-          <t>250014820</t>
+          <t>250009233</t>
         </is>
       </c>
       <c r="O52" t="inlineStr">
         <is>
-          <t>250014820</t>
+          <t>250009233</t>
         </is>
       </c>
       <c r="P52" t="inlineStr"/>
@@ -3639,27 +3639,27 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>33339916837</t>
+          <t>90111249104</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>CONTROLE A PLUS - SP 24,99</t>
+          <t>TIM CONTROLE A PLUS - 29,99</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>24,99</t>
+          <t>29,99</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>11963325952</t>
+          <t>94984485952</t>
         </is>
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>11983885820</t>
+          <t>94981705275</t>
         </is>
       </c>
       <c r="F53" t="inlineStr"/>
@@ -3667,12 +3667,12 @@
       <c r="H53" t="inlineStr"/>
       <c r="I53" t="inlineStr">
         <is>
-          <t>1-1695351555314</t>
+          <t>1-1685815276591</t>
         </is>
       </c>
       <c r="J53" t="inlineStr">
         <is>
-          <t>1-1695351555314</t>
+          <t>1-1685815276591</t>
         </is>
       </c>
       <c r="K53" t="inlineStr"/>
@@ -3680,12 +3680,12 @@
       <c r="M53" t="inlineStr"/>
       <c r="N53" t="inlineStr">
         <is>
-          <t>250014637</t>
+          <t>250009301</t>
         </is>
       </c>
       <c r="O53" t="inlineStr">
         <is>
-          <t>250014637</t>
+          <t>250009301</t>
         </is>
       </c>
       <c r="P53" t="inlineStr"/>
@@ -3700,27 +3700,27 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>96756012134</t>
+          <t>42071097068</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>TIM CONTROLE A PLUS - 29,99</t>
+          <t>TIM CONTROLE A PLUS - 31,99</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>29,99</t>
+          <t>31,99</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>62994097709</t>
+          <t>51991582189</t>
         </is>
       </c>
       <c r="E54" t="inlineStr">
         <is>
-          <t>62984452963</t>
+          <t>51981621590</t>
         </is>
       </c>
       <c r="F54" t="inlineStr"/>
@@ -3728,12 +3728,12 @@
       <c r="H54" t="inlineStr"/>
       <c r="I54" t="inlineStr">
         <is>
-          <t>1-1695324180440</t>
+          <t>1-1685610072003</t>
         </is>
       </c>
       <c r="J54" t="inlineStr">
         <is>
-          <t>1-1695324180440</t>
+          <t>1-1685610072003</t>
         </is>
       </c>
       <c r="K54" t="inlineStr"/>
@@ -3741,12 +3741,12 @@
       <c r="M54" t="inlineStr"/>
       <c r="N54" t="inlineStr">
         <is>
-          <t>250014605</t>
+          <t>250009010</t>
         </is>
       </c>
       <c r="O54" t="inlineStr">
         <is>
-          <t>250014605</t>
+          <t>250009010</t>
         </is>
       </c>
       <c r="P54" t="inlineStr"/>
@@ -3761,7 +3761,7 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>00714382540</t>
+          <t>10853595739</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
@@ -3776,12 +3776,12 @@
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>73999229032</t>
+          <t>21997996823</t>
         </is>
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>73991865156</t>
+          <t>21981654038</t>
         </is>
       </c>
       <c r="F55" t="inlineStr"/>
@@ -3789,12 +3789,12 @@
       <c r="H55" t="inlineStr"/>
       <c r="I55" t="inlineStr">
         <is>
-          <t>1-1695324182296</t>
+          <t>1-1699966597543</t>
         </is>
       </c>
       <c r="J55" t="inlineStr">
         <is>
-          <t>1-1695324182296</t>
+          <t>1-1699966597543</t>
         </is>
       </c>
       <c r="K55" t="inlineStr"/>
@@ -3802,12 +3802,12 @@
       <c r="M55" t="inlineStr"/>
       <c r="N55" t="inlineStr">
         <is>
-          <t>250014607</t>
+          <t>250009126</t>
         </is>
       </c>
       <c r="O55" t="inlineStr">
         <is>
-          <t>250014607</t>
+          <t>250009126</t>
         </is>
       </c>
       <c r="P55" t="inlineStr"/>
@@ -3822,27 +3822,27 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>10999134620</t>
+          <t>29643387879</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>TIM CONTROLE A PLUS - 31,99</t>
+          <t>TIM CONTROLE A PLUS - 29,99</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>31,99</t>
+          <t>29,99</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>33999028507</t>
+          <t>11977815463</t>
         </is>
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>33991695955</t>
+          <t>11981446172</t>
         </is>
       </c>
       <c r="F56" t="inlineStr"/>
@@ -3850,12 +3850,12 @@
       <c r="H56" t="inlineStr"/>
       <c r="I56" t="inlineStr">
         <is>
-          <t>1-1695139417921</t>
+          <t>1-1685424548922</t>
         </is>
       </c>
       <c r="J56" t="inlineStr">
         <is>
-          <t>1-1695139417921</t>
+          <t>1-1685424548922</t>
         </is>
       </c>
       <c r="K56" t="inlineStr"/>
@@ -3863,12 +3863,12 @@
       <c r="M56" t="inlineStr"/>
       <c r="N56" t="inlineStr">
         <is>
-          <t>250014558</t>
+          <t>250008820</t>
         </is>
       </c>
       <c r="O56" t="inlineStr">
         <is>
-          <t>250014558</t>
+          <t>250008820</t>
         </is>
       </c>
       <c r="P56" t="inlineStr"/>
@@ -3883,27 +3883,27 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>32494347874</t>
+          <t>26421089615</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>TIM CONTROLE SMART - DESC 43 - 46,99</t>
+          <t>TIM CONTROLE A PLUS - 31,99</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>46,99</t>
+          <t>31,99</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>11974415725</t>
+          <t>31995071905</t>
         </is>
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>11983884334</t>
+          <t>31991127748</t>
         </is>
       </c>
       <c r="F57" t="inlineStr"/>
@@ -3911,12 +3911,12 @@
       <c r="H57" t="inlineStr"/>
       <c r="I57" t="inlineStr">
         <is>
-          <t>1-1695068034304</t>
+          <t>1-1685456404946</t>
         </is>
       </c>
       <c r="J57" t="inlineStr">
         <is>
-          <t>1-1695068034304</t>
+          <t>1-1685456404946</t>
         </is>
       </c>
       <c r="K57" t="inlineStr"/>
@@ -3924,12 +3924,12 @@
       <c r="M57" t="inlineStr"/>
       <c r="N57" t="inlineStr">
         <is>
-          <t>250014505</t>
+          <t>250008836</t>
         </is>
       </c>
       <c r="O57" t="inlineStr">
         <is>
-          <t>250014505</t>
+          <t>250008836</t>
         </is>
       </c>
       <c r="P57" t="inlineStr"/>
@@ -3944,7 +3944,7 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>30777739615</t>
+          <t>45039530870</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
@@ -3959,12 +3959,12 @@
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>33984285910</t>
+          <t>11944400689</t>
         </is>
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>33991486876</t>
+          <t>11981452187</t>
         </is>
       </c>
       <c r="F58" t="inlineStr"/>
@@ -3972,12 +3972,12 @@
       <c r="H58" t="inlineStr"/>
       <c r="I58" t="inlineStr">
         <is>
-          <t>1-1695149109351</t>
+          <t>1-1685428859465</t>
         </is>
       </c>
       <c r="J58" t="inlineStr">
         <is>
-          <t>1-1695149109351</t>
+          <t>1-1685428859465</t>
         </is>
       </c>
       <c r="K58" t="inlineStr"/>
@@ -3985,12 +3985,12 @@
       <c r="M58" t="inlineStr"/>
       <c r="N58" t="inlineStr">
         <is>
-          <t>250014570</t>
+          <t>250008850</t>
         </is>
       </c>
       <c r="O58" t="inlineStr">
         <is>
-          <t>250014570</t>
+          <t>250008850</t>
         </is>
       </c>
       <c r="P58" t="inlineStr"/>
@@ -4005,7 +4005,7 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>36980270893</t>
+          <t>27721838827</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
@@ -4020,12 +4020,12 @@
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>17991326935</t>
+          <t>11962759994</t>
         </is>
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>17981484267</t>
+          <t>11981431949</t>
         </is>
       </c>
       <c r="F59" t="inlineStr"/>
@@ -4033,12 +4033,12 @@
       <c r="H59" t="inlineStr"/>
       <c r="I59" t="inlineStr">
         <is>
-          <t>1-1695162177188</t>
+          <t>1-1685252647243</t>
         </is>
       </c>
       <c r="J59" t="inlineStr">
         <is>
-          <t>1-1695162177188</t>
+          <t>1-1685252647243</t>
         </is>
       </c>
       <c r="K59" t="inlineStr"/>
@@ -4046,12 +4046,12 @@
       <c r="M59" t="inlineStr"/>
       <c r="N59" t="inlineStr">
         <is>
-          <t>250014559</t>
+          <t>250008767</t>
         </is>
       </c>
       <c r="O59" t="inlineStr">
         <is>
-          <t>250014559</t>
+          <t>250008767</t>
         </is>
       </c>
       <c r="P59" t="inlineStr"/>
@@ -4066,7 +4066,7 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>37960471819</t>
+          <t>70397690690</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
@@ -4081,12 +4081,12 @@
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>16997633181</t>
+          <t>38999069483</t>
         </is>
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>16981360729</t>
+          <t>38991986540</t>
         </is>
       </c>
       <c r="F60" t="inlineStr"/>
@@ -4094,12 +4094,12 @@
       <c r="H60" t="inlineStr"/>
       <c r="I60" t="inlineStr">
         <is>
-          <t>1-1694862736524</t>
+          <t>1-1702628809930</t>
         </is>
       </c>
       <c r="J60" t="inlineStr">
         <is>
-          <t>1-1694862736524</t>
+          <t>1-1702628809930</t>
         </is>
       </c>
       <c r="K60" t="inlineStr"/>
@@ -4107,12 +4107,12 @@
       <c r="M60" t="inlineStr"/>
       <c r="N60" t="inlineStr">
         <is>
-          <t>250014417</t>
+          <t>250008777</t>
         </is>
       </c>
       <c r="O60" t="inlineStr">
         <is>
-          <t>250014417</t>
+          <t>250008777</t>
         </is>
       </c>
       <c r="P60" t="inlineStr"/>
@@ -4127,27 +4127,27 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>75430150800</t>
+          <t>84031891253</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>TIM CONTROLE A PLUS - 31,99</t>
+          <t>TIM CONTROLE A PLUS - 29,99</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>31,99</t>
+          <t>29,99</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>17991417569</t>
+          <t>93991714634</t>
         </is>
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>17981549577</t>
+          <t>93981201394</t>
         </is>
       </c>
       <c r="F61" t="inlineStr"/>
@@ -4155,12 +4155,12 @@
       <c r="H61" t="inlineStr"/>
       <c r="I61" t="inlineStr">
         <is>
-          <t>1-1694553838607</t>
+          <t>1-1685046113166</t>
         </is>
       </c>
       <c r="J61" t="inlineStr">
         <is>
-          <t>1-1694553838607</t>
+          <t>1-1685046113166</t>
         </is>
       </c>
       <c r="K61" t="inlineStr"/>
@@ -4168,12 +4168,12 @@
       <c r="M61" t="inlineStr"/>
       <c r="N61" t="inlineStr">
         <is>
-          <t>250014318</t>
+          <t>250008476</t>
         </is>
       </c>
       <c r="O61" t="inlineStr">
         <is>
-          <t>250014318</t>
+          <t>250008476</t>
         </is>
       </c>
       <c r="P61" t="inlineStr"/>
@@ -4188,7 +4188,7 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>11473208963</t>
+          <t>00221917713</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
@@ -4203,38 +4203,30 @@
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>44974003498</t>
+          <t>22998762333</t>
         </is>
       </c>
       <c r="E62" t="inlineStr">
         <is>
-          <t>44999783545</t>
+          <t>22988075138</t>
         </is>
       </c>
       <c r="F62" t="inlineStr"/>
       <c r="G62" t="inlineStr"/>
       <c r="H62" t="inlineStr"/>
-      <c r="I62" t="inlineStr">
-        <is>
-          <t>1-1694082679009</t>
-        </is>
-      </c>
-      <c r="J62" t="inlineStr">
-        <is>
-          <t>1-1694082679009</t>
-        </is>
-      </c>
+      <c r="I62" t="inlineStr"/>
+      <c r="J62" t="inlineStr"/>
       <c r="K62" t="inlineStr"/>
       <c r="L62" t="inlineStr"/>
       <c r="M62" t="inlineStr"/>
       <c r="N62" t="inlineStr">
         <is>
-          <t>250014169</t>
+          <t>250008248</t>
         </is>
       </c>
       <c r="O62" t="inlineStr">
         <is>
-          <t>250014169</t>
+          <t>250008248</t>
         </is>
       </c>
       <c r="P62" t="inlineStr"/>
@@ -4246,6 +4238,1043 @@
         </is>
       </c>
     </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>13392095788</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>TIM CONTROLE A PLUS - 31,99</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>31,99</t>
+        </is>
+      </c>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>27992335359</t>
+        </is>
+      </c>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>27981164922</t>
+        </is>
+      </c>
+      <c r="F63" t="inlineStr"/>
+      <c r="G63" t="inlineStr"/>
+      <c r="H63" t="inlineStr"/>
+      <c r="I63" t="inlineStr">
+        <is>
+          <t>1-1684819211657</t>
+        </is>
+      </c>
+      <c r="J63" t="inlineStr">
+        <is>
+          <t>1-1684819211657</t>
+        </is>
+      </c>
+      <c r="K63" t="inlineStr"/>
+      <c r="L63" t="inlineStr"/>
+      <c r="M63" t="inlineStr"/>
+      <c r="N63" t="inlineStr">
+        <is>
+          <t>250008157</t>
+        </is>
+      </c>
+      <c r="O63" t="inlineStr">
+        <is>
+          <t>250008157</t>
+        </is>
+      </c>
+      <c r="P63" t="inlineStr"/>
+      <c r="Q63" t="inlineStr"/>
+      <c r="R63" t="inlineStr"/>
+      <c r="S63" t="inlineStr">
+        <is>
+          <t>Status Cancelado</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>81855451115</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>TIM CONTROLE A PLUS - 29,99</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>29,99</t>
+        </is>
+      </c>
+      <c r="D64" t="inlineStr">
+        <is>
+          <t>61985657819</t>
+        </is>
+      </c>
+      <c r="E64" t="inlineStr">
+        <is>
+          <t>61984122975</t>
+        </is>
+      </c>
+      <c r="F64" t="inlineStr"/>
+      <c r="G64" t="inlineStr"/>
+      <c r="H64" t="inlineStr"/>
+      <c r="I64" t="inlineStr">
+        <is>
+          <t>1-1684690922118</t>
+        </is>
+      </c>
+      <c r="J64" t="inlineStr">
+        <is>
+          <t>1-1684690922118</t>
+        </is>
+      </c>
+      <c r="K64" t="inlineStr"/>
+      <c r="L64" t="inlineStr"/>
+      <c r="M64" t="inlineStr"/>
+      <c r="N64" t="inlineStr">
+        <is>
+          <t>250007982</t>
+        </is>
+      </c>
+      <c r="O64" t="inlineStr">
+        <is>
+          <t>250007982</t>
+        </is>
+      </c>
+      <c r="P64" t="inlineStr"/>
+      <c r="Q64" t="inlineStr"/>
+      <c r="R64" t="inlineStr"/>
+      <c r="S64" t="inlineStr">
+        <is>
+          <t>Status Cancelado</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>62882279604</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>TIM CONTROLE A PLUS - 31,99</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>31,99</t>
+        </is>
+      </c>
+      <c r="D65" t="inlineStr">
+        <is>
+          <t>31984193028</t>
+        </is>
+      </c>
+      <c r="E65" t="inlineStr">
+        <is>
+          <t>31991064498</t>
+        </is>
+      </c>
+      <c r="F65" t="inlineStr"/>
+      <c r="G65" t="inlineStr"/>
+      <c r="H65" t="inlineStr"/>
+      <c r="I65" t="inlineStr">
+        <is>
+          <t>1-1684636376965</t>
+        </is>
+      </c>
+      <c r="J65" t="inlineStr">
+        <is>
+          <t>1-1684636376965</t>
+        </is>
+      </c>
+      <c r="K65" t="inlineStr"/>
+      <c r="L65" t="inlineStr"/>
+      <c r="M65" t="inlineStr"/>
+      <c r="N65" t="inlineStr">
+        <is>
+          <t>250007918</t>
+        </is>
+      </c>
+      <c r="O65" t="inlineStr">
+        <is>
+          <t>250007918</t>
+        </is>
+      </c>
+      <c r="P65" t="inlineStr"/>
+      <c r="Q65" t="inlineStr"/>
+      <c r="R65" t="inlineStr"/>
+      <c r="S65" t="inlineStr">
+        <is>
+          <t>Status Cancelado</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>50622498649</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>TIM CONTROLE A PLUS - 31,99</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>31,99</t>
+        </is>
+      </c>
+      <c r="D66" t="inlineStr">
+        <is>
+          <t>38997421908</t>
+        </is>
+      </c>
+      <c r="E66" t="inlineStr">
+        <is>
+          <t>38991986569</t>
+        </is>
+      </c>
+      <c r="F66" t="inlineStr"/>
+      <c r="G66" t="inlineStr"/>
+      <c r="H66" t="inlineStr"/>
+      <c r="I66" t="inlineStr">
+        <is>
+          <t>1-1702616132461</t>
+        </is>
+      </c>
+      <c r="J66" t="inlineStr">
+        <is>
+          <t>1-1702616132461</t>
+        </is>
+      </c>
+      <c r="K66" t="inlineStr"/>
+      <c r="L66" t="inlineStr"/>
+      <c r="M66" t="inlineStr"/>
+      <c r="N66" t="inlineStr">
+        <is>
+          <t>250007871</t>
+        </is>
+      </c>
+      <c r="O66" t="inlineStr">
+        <is>
+          <t>250007871</t>
+        </is>
+      </c>
+      <c r="P66" t="inlineStr"/>
+      <c r="Q66" t="inlineStr"/>
+      <c r="R66" t="inlineStr"/>
+      <c r="S66" t="inlineStr">
+        <is>
+          <t>Status Cancelado</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>03906494900</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>TIM CONTROLE A PLUS - 31,99</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>31,99</t>
+        </is>
+      </c>
+      <c r="D67" t="inlineStr">
+        <is>
+          <t>44988426795</t>
+        </is>
+      </c>
+      <c r="E67" t="inlineStr">
+        <is>
+          <t>44999032249</t>
+        </is>
+      </c>
+      <c r="F67" t="inlineStr"/>
+      <c r="G67" t="inlineStr"/>
+      <c r="H67" t="inlineStr"/>
+      <c r="I67" t="inlineStr">
+        <is>
+          <t>1-1684606933036</t>
+        </is>
+      </c>
+      <c r="J67" t="inlineStr">
+        <is>
+          <t>1-1684606933036</t>
+        </is>
+      </c>
+      <c r="K67" t="inlineStr"/>
+      <c r="L67" t="inlineStr"/>
+      <c r="M67" t="inlineStr"/>
+      <c r="N67" t="inlineStr">
+        <is>
+          <t>250007858</t>
+        </is>
+      </c>
+      <c r="O67" t="inlineStr">
+        <is>
+          <t>250007858</t>
+        </is>
+      </c>
+      <c r="P67" t="inlineStr"/>
+      <c r="Q67" t="inlineStr"/>
+      <c r="R67" t="inlineStr"/>
+      <c r="S67" t="inlineStr">
+        <is>
+          <t>Status Cancelado</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>33101202876</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>TIM CONTROLE A PLUS - 31,99</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>31,99</t>
+        </is>
+      </c>
+      <c r="D68" t="inlineStr">
+        <is>
+          <t>11978614051</t>
+        </is>
+      </c>
+      <c r="E68" t="inlineStr">
+        <is>
+          <t>11986098627</t>
+        </is>
+      </c>
+      <c r="F68" t="inlineStr"/>
+      <c r="G68" t="inlineStr"/>
+      <c r="H68" t="inlineStr"/>
+      <c r="I68" t="inlineStr">
+        <is>
+          <t>1-1684186329613</t>
+        </is>
+      </c>
+      <c r="J68" t="inlineStr">
+        <is>
+          <t>1-1684186329613</t>
+        </is>
+      </c>
+      <c r="K68" t="inlineStr"/>
+      <c r="L68" t="inlineStr"/>
+      <c r="M68" t="inlineStr"/>
+      <c r="N68" t="inlineStr">
+        <is>
+          <t>250007508</t>
+        </is>
+      </c>
+      <c r="O68" t="inlineStr">
+        <is>
+          <t>250007508</t>
+        </is>
+      </c>
+      <c r="P68" t="inlineStr"/>
+      <c r="Q68" t="inlineStr"/>
+      <c r="R68" t="inlineStr"/>
+      <c r="S68" t="inlineStr">
+        <is>
+          <t>Status Cancelado</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>10061008656</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>TIM CONTROLE A PLUS - 29,99</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>29,99</t>
+        </is>
+      </c>
+      <c r="D69" t="inlineStr">
+        <is>
+          <t>35998877685</t>
+        </is>
+      </c>
+      <c r="E69" t="inlineStr">
+        <is>
+          <t>35991390745</t>
+        </is>
+      </c>
+      <c r="F69" t="inlineStr"/>
+      <c r="G69" t="inlineStr"/>
+      <c r="H69" t="inlineStr"/>
+      <c r="I69" t="inlineStr">
+        <is>
+          <t>1-1683975123284</t>
+        </is>
+      </c>
+      <c r="J69" t="inlineStr">
+        <is>
+          <t>1-1683975123284</t>
+        </is>
+      </c>
+      <c r="K69" t="inlineStr"/>
+      <c r="L69" t="inlineStr"/>
+      <c r="M69" t="inlineStr"/>
+      <c r="N69" t="inlineStr">
+        <is>
+          <t>250007216</t>
+        </is>
+      </c>
+      <c r="O69" t="inlineStr">
+        <is>
+          <t>250007216</t>
+        </is>
+      </c>
+      <c r="P69" t="inlineStr"/>
+      <c r="Q69" t="inlineStr"/>
+      <c r="R69" t="inlineStr"/>
+      <c r="S69" t="inlineStr">
+        <is>
+          <t>Status Cancelado</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>67844340487</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>TIM CONTROLE A PLUS - 29,99</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>29,99</t>
+        </is>
+      </c>
+      <c r="D70" t="inlineStr">
+        <is>
+          <t>82993725326</t>
+        </is>
+      </c>
+      <c r="E70" t="inlineStr">
+        <is>
+          <t>82996654991</t>
+        </is>
+      </c>
+      <c r="F70" t="inlineStr"/>
+      <c r="G70" t="inlineStr"/>
+      <c r="H70" t="inlineStr"/>
+      <c r="I70" t="inlineStr">
+        <is>
+          <t>1-1684001775168</t>
+        </is>
+      </c>
+      <c r="J70" t="inlineStr">
+        <is>
+          <t>1-1684001775168</t>
+        </is>
+      </c>
+      <c r="K70" t="inlineStr"/>
+      <c r="L70" t="inlineStr"/>
+      <c r="M70" t="inlineStr"/>
+      <c r="N70" t="inlineStr">
+        <is>
+          <t>250007223</t>
+        </is>
+      </c>
+      <c r="O70" t="inlineStr">
+        <is>
+          <t>250007223</t>
+        </is>
+      </c>
+      <c r="P70" t="inlineStr"/>
+      <c r="Q70" t="inlineStr"/>
+      <c r="R70" t="inlineStr"/>
+      <c r="S70" t="inlineStr">
+        <is>
+          <t>Status Cancelado</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>02260591469</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>TIM CONTROLE A PLUS - 29,99</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>29,99</t>
+        </is>
+      </c>
+      <c r="D71" t="inlineStr">
+        <is>
+          <t>81993170153</t>
+        </is>
+      </c>
+      <c r="E71" t="inlineStr">
+        <is>
+          <t>81996063795</t>
+        </is>
+      </c>
+      <c r="F71" t="inlineStr"/>
+      <c r="G71" t="inlineStr"/>
+      <c r="H71" t="inlineStr"/>
+      <c r="I71" t="inlineStr">
+        <is>
+          <t>1-1684082455126</t>
+        </is>
+      </c>
+      <c r="J71" t="inlineStr">
+        <is>
+          <t>1-1684082455126</t>
+        </is>
+      </c>
+      <c r="K71" t="inlineStr"/>
+      <c r="L71" t="inlineStr"/>
+      <c r="M71" t="inlineStr"/>
+      <c r="N71" t="inlineStr">
+        <is>
+          <t>250007356</t>
+        </is>
+      </c>
+      <c r="O71" t="inlineStr">
+        <is>
+          <t>250007356</t>
+        </is>
+      </c>
+      <c r="P71" t="inlineStr"/>
+      <c r="Q71" t="inlineStr"/>
+      <c r="R71" t="inlineStr"/>
+      <c r="S71" t="inlineStr">
+        <is>
+          <t>Status Cancelado</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>60286873249</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>TIM CONTROLE A PLUS - 29,99</t>
+        </is>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>29,99</t>
+        </is>
+      </c>
+      <c r="D72" t="inlineStr">
+        <is>
+          <t>92985991176</t>
+        </is>
+      </c>
+      <c r="E72" t="inlineStr">
+        <is>
+          <t>92982505922</t>
+        </is>
+      </c>
+      <c r="F72" t="inlineStr"/>
+      <c r="G72" t="inlineStr"/>
+      <c r="H72" t="inlineStr"/>
+      <c r="I72" t="inlineStr">
+        <is>
+          <t>1-1684016061607</t>
+        </is>
+      </c>
+      <c r="J72" t="inlineStr">
+        <is>
+          <t>1-1684016061607</t>
+        </is>
+      </c>
+      <c r="K72" t="inlineStr"/>
+      <c r="L72" t="inlineStr"/>
+      <c r="M72" t="inlineStr"/>
+      <c r="N72" t="inlineStr">
+        <is>
+          <t>250007279</t>
+        </is>
+      </c>
+      <c r="O72" t="inlineStr">
+        <is>
+          <t>250007279</t>
+        </is>
+      </c>
+      <c r="P72" t="inlineStr"/>
+      <c r="Q72" t="inlineStr"/>
+      <c r="R72" t="inlineStr"/>
+      <c r="S72" t="inlineStr">
+        <is>
+          <t>Status Cancelado</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>03610176857</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>TIM CONTROLE A PLUS - 29,99</t>
+        </is>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>29,99</t>
+        </is>
+      </c>
+      <c r="D73" t="inlineStr">
+        <is>
+          <t>11997569002</t>
+        </is>
+      </c>
+      <c r="E73" t="inlineStr">
+        <is>
+          <t>11986860516</t>
+        </is>
+      </c>
+      <c r="F73" t="inlineStr"/>
+      <c r="G73" t="inlineStr"/>
+      <c r="H73" t="inlineStr"/>
+      <c r="I73" t="inlineStr">
+        <is>
+          <t>1-1683998723745</t>
+        </is>
+      </c>
+      <c r="J73" t="inlineStr">
+        <is>
+          <t>1-1683998723745</t>
+        </is>
+      </c>
+      <c r="K73" t="inlineStr"/>
+      <c r="L73" t="inlineStr"/>
+      <c r="M73" t="inlineStr"/>
+      <c r="N73" t="inlineStr">
+        <is>
+          <t>250007244</t>
+        </is>
+      </c>
+      <c r="O73" t="inlineStr">
+        <is>
+          <t>250007244</t>
+        </is>
+      </c>
+      <c r="P73" t="inlineStr"/>
+      <c r="Q73" t="inlineStr"/>
+      <c r="R73" t="inlineStr"/>
+      <c r="S73" t="inlineStr">
+        <is>
+          <t>Status Cancelado</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>29679589803</t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>TIM CONTROLE A PLUS - 31,99</t>
+        </is>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>31,99</t>
+        </is>
+      </c>
+      <c r="D74" t="inlineStr">
+        <is>
+          <t>19995591369</t>
+        </is>
+      </c>
+      <c r="E74" t="inlineStr">
+        <is>
+          <t>19982033115</t>
+        </is>
+      </c>
+      <c r="F74" t="inlineStr"/>
+      <c r="G74" t="inlineStr"/>
+      <c r="H74" t="inlineStr"/>
+      <c r="I74" t="inlineStr">
+        <is>
+          <t>1-1684278010829</t>
+        </is>
+      </c>
+      <c r="J74" t="inlineStr">
+        <is>
+          <t>1-1684278010829</t>
+        </is>
+      </c>
+      <c r="K74" t="inlineStr"/>
+      <c r="L74" t="inlineStr"/>
+      <c r="M74" t="inlineStr"/>
+      <c r="N74" t="inlineStr">
+        <is>
+          <t>250007158</t>
+        </is>
+      </c>
+      <c r="O74" t="inlineStr">
+        <is>
+          <t>250007158</t>
+        </is>
+      </c>
+      <c r="P74" t="inlineStr"/>
+      <c r="Q74" t="inlineStr"/>
+      <c r="R74" t="inlineStr"/>
+      <c r="S74" t="inlineStr">
+        <is>
+          <t>Status Cancelado</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>47075376004</t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>TIM CONTROLE A PLUS - 29,99</t>
+        </is>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>29,99</t>
+        </is>
+      </c>
+      <c r="D75" t="inlineStr">
+        <is>
+          <t>51981771953</t>
+        </is>
+      </c>
+      <c r="E75" t="inlineStr">
+        <is>
+          <t>51981759188</t>
+        </is>
+      </c>
+      <c r="F75" t="inlineStr"/>
+      <c r="G75" t="inlineStr"/>
+      <c r="H75" t="inlineStr"/>
+      <c r="I75" t="inlineStr">
+        <is>
+          <t>1-1697556265173</t>
+        </is>
+      </c>
+      <c r="J75" t="inlineStr">
+        <is>
+          <t>1-1697556265173</t>
+        </is>
+      </c>
+      <c r="K75" t="inlineStr"/>
+      <c r="L75" t="inlineStr"/>
+      <c r="M75" t="inlineStr"/>
+      <c r="N75" t="inlineStr">
+        <is>
+          <t>250007182</t>
+        </is>
+      </c>
+      <c r="O75" t="inlineStr">
+        <is>
+          <t>250007182</t>
+        </is>
+      </c>
+      <c r="P75" t="inlineStr"/>
+      <c r="Q75" t="inlineStr"/>
+      <c r="R75" t="inlineStr"/>
+      <c r="S75" t="inlineStr">
+        <is>
+          <t>Status Cancelado</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>32010695828</t>
+        </is>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>TIM CONTROLE A PLUS - 29,99</t>
+        </is>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>29,99</t>
+        </is>
+      </c>
+      <c r="D76" t="inlineStr">
+        <is>
+          <t>44988368126</t>
+        </is>
+      </c>
+      <c r="E76" t="inlineStr">
+        <is>
+          <t>44999053769</t>
+        </is>
+      </c>
+      <c r="F76" t="inlineStr"/>
+      <c r="G76" t="inlineStr"/>
+      <c r="H76" t="inlineStr"/>
+      <c r="I76" t="inlineStr">
+        <is>
+          <t>1-1683857617154</t>
+        </is>
+      </c>
+      <c r="J76" t="inlineStr">
+        <is>
+          <t>1-1683857617154</t>
+        </is>
+      </c>
+      <c r="K76" t="inlineStr"/>
+      <c r="L76" t="inlineStr"/>
+      <c r="M76" t="inlineStr"/>
+      <c r="N76" t="inlineStr">
+        <is>
+          <t>250007077</t>
+        </is>
+      </c>
+      <c r="O76" t="inlineStr">
+        <is>
+          <t>250007077</t>
+        </is>
+      </c>
+      <c r="P76" t="inlineStr"/>
+      <c r="Q76" t="inlineStr"/>
+      <c r="R76" t="inlineStr"/>
+      <c r="S76" t="inlineStr">
+        <is>
+          <t>Status Cancelado</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>56633637268</t>
+        </is>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>TIM CONTROLE A PLUS - 29,99</t>
+        </is>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>29,99</t>
+        </is>
+      </c>
+      <c r="D77" t="inlineStr">
+        <is>
+          <t>69992049995</t>
+        </is>
+      </c>
+      <c r="E77" t="inlineStr">
+        <is>
+          <t>69981686113</t>
+        </is>
+      </c>
+      <c r="F77" t="inlineStr"/>
+      <c r="G77" t="inlineStr"/>
+      <c r="H77" t="inlineStr"/>
+      <c r="I77" t="inlineStr">
+        <is>
+          <t>1-1683849279260</t>
+        </is>
+      </c>
+      <c r="J77" t="inlineStr">
+        <is>
+          <t>1-1683849279260</t>
+        </is>
+      </c>
+      <c r="K77" t="inlineStr"/>
+      <c r="L77" t="inlineStr"/>
+      <c r="M77" t="inlineStr"/>
+      <c r="N77" t="inlineStr">
+        <is>
+          <t>250007040</t>
+        </is>
+      </c>
+      <c r="O77" t="inlineStr">
+        <is>
+          <t>250007040</t>
+        </is>
+      </c>
+      <c r="P77" t="inlineStr"/>
+      <c r="Q77" t="inlineStr"/>
+      <c r="R77" t="inlineStr"/>
+      <c r="S77" t="inlineStr">
+        <is>
+          <t>Status Cancelado</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>00517037505</t>
+        </is>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>TIM CONTROLE A PLUS - 29,99</t>
+        </is>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>29,99</t>
+        </is>
+      </c>
+      <c r="D78" t="inlineStr">
+        <is>
+          <t>75983455050</t>
+        </is>
+      </c>
+      <c r="E78" t="inlineStr">
+        <is>
+          <t>75991760206</t>
+        </is>
+      </c>
+      <c r="F78" t="inlineStr"/>
+      <c r="G78" t="inlineStr"/>
+      <c r="H78" t="inlineStr"/>
+      <c r="I78" t="inlineStr">
+        <is>
+          <t>1-1691787745183</t>
+        </is>
+      </c>
+      <c r="J78" t="inlineStr">
+        <is>
+          <t>1-1691787745183</t>
+        </is>
+      </c>
+      <c r="K78" t="inlineStr"/>
+      <c r="L78" t="inlineStr"/>
+      <c r="M78" t="inlineStr"/>
+      <c r="N78" t="inlineStr">
+        <is>
+          <t>250007138</t>
+        </is>
+      </c>
+      <c r="O78" t="inlineStr">
+        <is>
+          <t>250007138</t>
+        </is>
+      </c>
+      <c r="P78" t="inlineStr"/>
+      <c r="Q78" t="inlineStr"/>
+      <c r="R78" t="inlineStr"/>
+      <c r="S78" t="inlineStr">
+        <is>
+          <t>Status Cancelado</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>81027370500</t>
+        </is>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>TIM CONTROLE A PLUS - 29,99</t>
+        </is>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>29,99</t>
+        </is>
+      </c>
+      <c r="D79" t="inlineStr">
+        <is>
+          <t>79996067549</t>
+        </is>
+      </c>
+      <c r="E79" t="inlineStr">
+        <is>
+          <t>79991275890</t>
+        </is>
+      </c>
+      <c r="F79" t="inlineStr"/>
+      <c r="G79" t="inlineStr"/>
+      <c r="H79" t="inlineStr"/>
+      <c r="I79" t="inlineStr">
+        <is>
+          <t>1-1683851395639</t>
+        </is>
+      </c>
+      <c r="J79" t="inlineStr">
+        <is>
+          <t>1-1683851395639</t>
+        </is>
+      </c>
+      <c r="K79" t="inlineStr"/>
+      <c r="L79" t="inlineStr"/>
+      <c r="M79" t="inlineStr"/>
+      <c r="N79" t="inlineStr">
+        <is>
+          <t>250007048</t>
+        </is>
+      </c>
+      <c r="O79" t="inlineStr">
+        <is>
+          <t>250007048</t>
+        </is>
+      </c>
+      <c r="P79" t="inlineStr"/>
+      <c r="Q79" t="inlineStr"/>
+      <c r="R79" t="inlineStr"/>
+      <c r="S79" t="inlineStr">
+        <is>
+          <t>Status Cancelado</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>